<commit_message>
Created backlog for Sprint 2
</commit_message>
<xml_diff>
--- a/MealPlanner/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/MealPlanner/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westga365-my.sharepoint.com/personal/jcorley_westga_edu/Documents/Teaching/Software Engineering II/SE2 - Spring 2026/Project/SE2-project-repos-sample/sprints/sprint1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kirya\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{9C9C4265-351C-41A0-89E5-93A08D9C51A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C68B4513-1541-415B-8F23-00764467EF2F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D6FF39-01FA-4151-95A4-11A77EADC848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1110" yWindow="660" windowWidth="14565" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
   <si>
     <t>Related User Story</t>
   </si>
@@ -65,10 +65,58 @@
     <t>Estimate Totals</t>
   </si>
   <si>
-    <t>Code Things…</t>
-  </si>
-  <si>
-    <t>That User Story</t>
+    <t>Implement viewing planned meals</t>
+  </si>
+  <si>
+    <t>As a user I want to view planned meals so I can see what I have planned</t>
+  </si>
+  <si>
+    <t>Complete GroceryList</t>
+  </si>
+  <si>
+    <t>Basic Server Setup</t>
+  </si>
+  <si>
+    <t>View Meal (Server)</t>
+  </si>
+  <si>
+    <t>View Meal (Client)</t>
+  </si>
+  <si>
+    <t>Make Meal (Server)</t>
+  </si>
+  <si>
+    <t>Make Meal (Client)</t>
+  </si>
+  <si>
+    <t>Create Account (Server)</t>
+  </si>
+  <si>
+    <t>Create Account (Client)</t>
+  </si>
+  <si>
+    <t>Login (Server)</t>
+  </si>
+  <si>
+    <t>Login (Client)</t>
+  </si>
+  <si>
+    <t>As a user I want to generate a grocery list so that I can see what ingredients are necessary to make planned meals</t>
+  </si>
+  <si>
+    <t>As a user I want to have my planner information saved so I can access and use old information</t>
+  </si>
+  <si>
+    <t>As a user I want to be able to login so I can save  my information</t>
+  </si>
+  <si>
+    <t>As a user I want to be able to create an account so I can log in</t>
+  </si>
+  <si>
+    <t>As a user I want to make meal so I can add it to my planner</t>
+  </si>
+  <si>
+    <t>As a user I want to see what meals I have planned</t>
   </si>
 </sst>
 </file>
@@ -142,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -156,6 +204,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -314,16 +365,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>100</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>100</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>100</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1407,15 +1458,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C3" s="1">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="D3" s="2">
         <v>25</v>
@@ -1430,91 +1481,151 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
+    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
+    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3</v>
+      </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3</v>
+      </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="1">
+        <v>3</v>
+      </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
+    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1">
+        <v>3</v>
+      </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="1">
+        <v>3</v>
+      </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="1">
+        <v>3</v>
+      </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="1">
+        <v>3</v>
+      </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="A12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="1">
+        <v>3</v>
+      </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="A13" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="1">
+        <v>3</v>
+      </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -1643,7 +1754,7 @@
       </c>
       <c r="C27" s="3">
         <f>SUM(C3:C26)</f>
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="D27" s="3">
         <f t="shared" ref="D27:G27" si="0">SUM(D3:D26)</f>
@@ -1665,19 +1776,19 @@
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D28">
         <f>$C$27</f>
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="E28">
         <f t="shared" ref="E28:G28" si="1">$C$27</f>
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="F28">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="G28">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated appropriate documentation - Added Hour Enumeration to class diagram and its relation to the Planner class - Updated planner class' properties and methods
</commit_message>
<xml_diff>
--- a/MealPlanner/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/MealPlanner/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kirya\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a648f88e637c48b0/Coding Stuff/School/Software Engineering/Semester 2/Assignments/Group Project/MealPlanner/sprints/sprint2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D6FF39-01FA-4151-95A4-11A77EADC848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="13_ncr:1_{98D6FF39-01FA-4151-95A4-11A77EADC848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC19D213-82DF-4530-8470-8E5812484216}"/>
   <bookViews>
-    <workbookView xWindow="1110" yWindow="660" windowWidth="14565" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -59,9 +59,6 @@
     <t>Week 4</t>
   </si>
   <si>
-    <t>Amount Remaining After…</t>
-  </si>
-  <si>
     <t>Estimate Totals</t>
   </si>
   <si>
@@ -117,6 +114,9 @@
   </si>
   <si>
     <t>As a user I want to see what meals I have planned</t>
+  </si>
+  <si>
+    <t>Hours spent</t>
   </si>
 </sst>
 </file>
@@ -199,14 +199,14 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -322,16 +322,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>25</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>50</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>75</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>100</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1425,26 +1425,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="D1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
       <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
@@ -1459,34 +1459,34 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>10</v>
+      <c r="A3" s="6" t="s">
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
       </c>
       <c r="D3" s="2">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E3" s="2">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="G3" s="2">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>21</v>
+      <c r="A4" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="1">
         <v>2</v>
@@ -1497,11 +1497,11 @@
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>22</v>
+      <c r="A5" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" s="1">
         <v>3</v>
@@ -1512,11 +1512,11 @@
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>23</v>
+      <c r="A6" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6" s="1">
         <v>3</v>
@@ -1527,11 +1527,11 @@
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>23</v>
+      <c r="A7" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7" s="1">
         <v>3</v>
@@ -1542,11 +1542,11 @@
       <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>24</v>
+      <c r="A8" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" s="1">
         <v>3</v>
@@ -1557,11 +1557,11 @@
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>24</v>
+      <c r="A9" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9" s="1">
         <v>3</v>
@@ -1572,11 +1572,11 @@
       <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>25</v>
+      <c r="A10" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" s="1">
         <v>3</v>
@@ -1587,11 +1587,11 @@
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>25</v>
+      <c r="A11" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" s="1">
         <v>3</v>
@@ -1602,11 +1602,11 @@
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>26</v>
+      <c r="A12" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" s="1">
         <v>3</v>
@@ -1617,11 +1617,11 @@
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>26</v>
+      <c r="A13" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1">
         <v>3</v>
@@ -1750,7 +1750,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B27" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C27" s="3">
         <f>SUM(C3:C26)</f>
@@ -1758,19 +1758,19 @@
       </c>
       <c r="D27" s="3">
         <f t="shared" ref="D27:G27" si="0">SUM(D3:D26)</f>
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E27" s="3">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" si="0"/>
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="G27" s="3">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated sprint burnup chart
</commit_message>
<xml_diff>
--- a/MealPlanner/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/MealPlanner/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a648f88e637c48b0/Coding Stuff/School/Software Engineering/Semester 2/Assignments/Group Project/MealPlanner/sprints/sprint2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="96" documentId="13_ncr:1_{98D6FF39-01FA-4151-95A4-11A77EADC848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC19D213-82DF-4530-8470-8E5812484216}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="13_ncr:1_{98D6FF39-01FA-4151-95A4-11A77EADC848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2BC0C18-121F-416C-9111-CAA67546F950}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -325,7 +325,7 @@
                   <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1153,6 +1153,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1626,10 +1630,18 @@
       <c r="C13" s="1">
         <v>3</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2">
+        <v>2</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
@@ -1762,7 +1774,7 @@
       </c>
       <c r="E27" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Revert "main branch changes"
This reverts commit ea89488887b48dc37a37d05e6ddb153e2042e92b.
</commit_message>
<xml_diff>
--- a/MealPlanner/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/MealPlanner/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30002"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a648f88e637c48b0/Coding Stuff/School/Software Engineering/Semester 2/Assignments/Group Project/MealPlanner/sprints/sprint2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="100" documentId="13_ncr:1_{98D6FF39-01FA-4151-95A4-11A77EADC848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2BC0C18-121F-416C-9111-CAA67546F950}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C7C40FC-ADAF-42CE-8F25-23CD0A487BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,6 +47,9 @@
     <t>Initial Estimate</t>
   </si>
   <si>
+    <t>Hours spent</t>
+  </si>
+  <si>
     <t>Week 1</t>
   </si>
   <si>
@@ -59,71 +62,68 @@
     <t>Week 4</t>
   </si>
   <si>
+    <t>As a user I want to view planned meals so I can see what I have planned</t>
+  </si>
+  <si>
+    <t>Implement viewing planned meals</t>
+  </si>
+  <si>
+    <t>As a user I want to generate a grocery list so that I can see what ingredients are necessary to make planned meals</t>
+  </si>
+  <si>
+    <t>Complete GroceryList</t>
+  </si>
+  <si>
+    <t>As a user I want to have my planner information saved so I can access and use old information</t>
+  </si>
+  <si>
+    <t>Basic Server Setup</t>
+  </si>
+  <si>
+    <t>As a user I want to be able to login so I can save  my information</t>
+  </si>
+  <si>
+    <t>Login (Client)</t>
+  </si>
+  <si>
+    <t>Login (Server)</t>
+  </si>
+  <si>
+    <t>As a user I want to be able to create an account so I can log in</t>
+  </si>
+  <si>
+    <t>Create Account (Client)</t>
+  </si>
+  <si>
+    <t>Create Account (Server)</t>
+  </si>
+  <si>
+    <t>As a user I want to make meal so I can add it to my planner</t>
+  </si>
+  <si>
+    <t>Make Meal (Client)</t>
+  </si>
+  <si>
+    <t>Make Meal (Server)</t>
+  </si>
+  <si>
+    <t>As a user I want to see what meals I have planned</t>
+  </si>
+  <si>
+    <t>View Meal (Client)</t>
+  </si>
+  <si>
+    <t>View Meal (Server)</t>
+  </si>
+  <si>
     <t>Estimate Totals</t>
-  </si>
-  <si>
-    <t>Implement viewing planned meals</t>
-  </si>
-  <si>
-    <t>As a user I want to view planned meals so I can see what I have planned</t>
-  </si>
-  <si>
-    <t>Complete GroceryList</t>
-  </si>
-  <si>
-    <t>Basic Server Setup</t>
-  </si>
-  <si>
-    <t>View Meal (Server)</t>
-  </si>
-  <si>
-    <t>View Meal (Client)</t>
-  </si>
-  <si>
-    <t>Make Meal (Server)</t>
-  </si>
-  <si>
-    <t>Make Meal (Client)</t>
-  </si>
-  <si>
-    <t>Create Account (Server)</t>
-  </si>
-  <si>
-    <t>Create Account (Client)</t>
-  </si>
-  <si>
-    <t>Login (Server)</t>
-  </si>
-  <si>
-    <t>Login (Client)</t>
-  </si>
-  <si>
-    <t>As a user I want to generate a grocery list so that I can see what ingredients are necessary to make planned meals</t>
-  </si>
-  <si>
-    <t>As a user I want to have my planner information saved so I can access and use old information</t>
-  </si>
-  <si>
-    <t>As a user I want to be able to login so I can save  my information</t>
-  </si>
-  <si>
-    <t>As a user I want to be able to create an account so I can log in</t>
-  </si>
-  <si>
-    <t>As a user I want to make meal so I can add it to my planner</t>
-  </si>
-  <si>
-    <t>As a user I want to see what meals I have planned</t>
-  </si>
-  <si>
-    <t>Hours spent</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -322,16 +322,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>5</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1153,10 +1153,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1421,14 +1417,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="51.42578125" customWidth="1"/>
     <col min="2" max="2" width="41.7109375" customWidth="1"/>
     <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1439,35 +1435,35 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
       <c r="D2" s="5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="30">
       <c r="A3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
@@ -1476,21 +1472,21 @@
         <v>5</v>
       </c>
       <c r="E3" s="2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F3" s="2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G3" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="45">
       <c r="A4" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" s="1">
         <v>2</v>
@@ -1500,87 +1496,127 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="30">
       <c r="A5" s="6" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1">
         <v>3</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="D5" s="2">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2">
+        <v>3</v>
+      </c>
+      <c r="F5" s="2">
+        <v>3</v>
+      </c>
+      <c r="G5" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30">
       <c r="A6" s="6" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1">
         <v>3</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>2</v>
+      </c>
+      <c r="G6" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="30">
       <c r="A7" s="6" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C7" s="1">
         <v>3</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>2</v>
+      </c>
+      <c r="F7" s="2">
+        <v>2</v>
+      </c>
+      <c r="G7" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30">
       <c r="A8" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1">
         <v>3</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2">
+        <v>2</v>
+      </c>
+      <c r="G8" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="30">
       <c r="A9" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C9" s="1">
         <v>3</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>2</v>
+      </c>
+      <c r="F9" s="2">
+        <v>2</v>
+      </c>
+      <c r="G9" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30">
       <c r="A10" s="6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C10" s="1">
         <v>3</v>
@@ -1590,12 +1626,12 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="30">
       <c r="A11" s="6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1">
         <v>3</v>
@@ -1605,12 +1641,12 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="A12" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1">
         <v>3</v>
@@ -1620,12 +1656,12 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="A13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="C13" s="1">
         <v>3</v>
@@ -1643,7 +1679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1652,7 +1688,7 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1661,7 +1697,7 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -1670,7 +1706,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1679,7 +1715,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1688,7 +1724,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1697,7 +1733,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1706,7 +1742,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1715,7 +1751,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1724,7 +1760,7 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1733,7 +1769,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1742,7 +1778,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1751,7 +1787,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1760,9 +1796,9 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7">
       <c r="B27" s="4" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="C27" s="3">
         <f>SUM(C3:C26)</f>
@@ -1770,22 +1806,22 @@
       </c>
       <c r="D27" s="3">
         <f t="shared" ref="D27:G27" si="0">SUM(D3:D26)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E27" s="3">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G27" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="D28">
         <f>$C$27</f>
         <v>32</v>

</xml_diff>